<commit_message>
rover_platform_mbse: follow the topic renames
The SWRS seeds, the SWRS_BAT/HWI/SAF/TRN sets (Description, Summary, AcceptanceCriteria,
Comments) and platform_architecture.json use hardware_interface/driver_state,
battery/battery_status, battery/charging_status and battery_udp_data. The two architecture ports
named after a topic follow (driver_state, battery_udp_data), and the battery remap citation
moves to rover_battery.launch.py:72.

Regenerated with build_all. The SysML export differs only by the renames once the allocation
numbering, which the exporter reshuffles on every build, is ignored. It passes the Pilot kernel.
Model tests: 25 passed, 7 known deviations, 0 unexpected. Traceability: 0 errors. The xlsx
exports whose cells changed are included (BAT, HWI, SAF, TRN SWRS and the SYS-SR compliance
workbook).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rover_platform_mbse/export/ROVER-A1-ROVER_BATTERY-SWRS-V-001.xlsx
+++ b/rover_platform_mbse/export/ROVER-A1-ROVER_BATTERY-SWRS-V-001.xlsx
@@ -570,7 +570,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>The rover_battery shall subscribe udp_msgs/UdpPacket on rover_battery_udp_data (depth 100), fed by the rover_udp_battery_receiver_node bound to ip 192.168.1.201, port 4444.</t>
+          <t>The rover_battery shall subscribe udp_msgs/UdpPacket on battery_udp_data (depth 100), fed by the rover_udp_battery_receiver_node bound to ip 192.168.1.201, port 4444.</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -585,7 +585,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>The launch-structure test finds the receiver and the battery node in one container with udp_read remapped to rover_battery_udp_data; the config has a section for each node.</t>
+          <t>The launch-structure test finds the receiver and the battery node in one container with udp_read remapped to battery_udp_data; the config has a section for each node.</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>The rover_battery shall publish sensor_msgs/BatteryState on rover_battery/battery_status (depth 5, reliable, volatile) once for every valid BMS frame received.</t>
+          <t>The rover_battery shall publish sensor_msgs/BatteryState on battery/battery_status (depth 5, reliable, volatile) once for every valid BMS frame received.</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -713,7 +713,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Each valid packet injected on rover_battery_udp_data produces exactly one BatteryState message.</t>
+          <t>Each valid packet injected on battery_udp_data produces exactly one BatteryState message.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>The rover_battery shall publish rover_msgs/ChargingStatus on rover_battery/charging_status (depth 5) with every battery state, with charging = (BMS status 1), current and current_battery = pack current, and charger_type WIRED while charging, UNKNOWN otherwise.</t>
+          <t>The rover_battery shall publish rover_msgs/ChargingStatus on battery/charging_status (depth 5) with every battery state, with charging = (BMS status 1), current and current_battery = pack current, and charger_type WIRED while charging, UNKNOWN otherwise.</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>The rover_battery shall publish rover_battery/battery_status at 1 Hz or faster regardless of the BMS packet timing, republishing the latest reading on a fixed-rate timer, and shall enter the watchdog state (SWR-BAT-008) when the latest reading is older than [TBD] s.</t>
+          <t>The rover_battery shall publish battery/battery_status at 1 Hz or faster regardless of the BMS packet timing, republishing the latest reading on a fixed-rate timer, and shall enter the watchdog state (SWR-BAT-008) when the latest reading is older than [TBD] s.</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>'ros2 topic hz rover_battery/battery_status' reports &gt;= 1 Hz with the BMS bridge sending at its nominal rate and with it silent (then carrying the watchdog state).</t>
+          <t>'ros2 topic hz battery/battery_status' reports &gt;= 1 Hz with the BMS bridge sending at its nominal rate and with it silent (then carrying the watchdog state).</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1612,7 +1612,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
@@ -1624,7 +1624,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>rover_battery decodes the Daly BMS telemetry that the ESP32 rover_led_bms_ble_controller forwards over UDP (392-byte payload, received by rover_udp_driver's UdpReceiverNode on 192.168.1.201:4444 in the same component container) and publishes the rover's battery state as sensor_msgs/BatteryState on rover_battery/battery_status and rover_msgs/ChargingStatus on rover_battery/charging_status, with a health classification from the BMS alarm bits, a data watchdog, and diagnostics. It is the battery input of rover_safety (battery E-Stop and shutdown policy, LED battery animations). State-of-charge thresholds live in the BMS configuration, not in this package.</t>
+          <t>rover_battery decodes the Daly BMS telemetry that the ESP32 rover_led_bms_ble_controller forwards over UDP (392-byte payload, received by rover_udp_driver's UdpReceiverNode on 192.168.1.201:4444 in the same component container) and publishes the rover's battery state as sensor_msgs/BatteryState on battery/battery_status and rover_msgs/ChargingStatus on battery/charging_status, with a health classification from the BMS alarm bits, a data watchdog, and diagnostics. It is the battery input of rover_safety (battery E-Stop and shutdown policy, LED battery animations). State-of-charge thresholds live in the BMS configuration, not in this package.</t>
         </is>
       </c>
     </row>
@@ -1726,7 +1726,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">

</xml_diff>